<commit_message>
Withdraw DPPO_CEON_0008, Component subclass-of Product
The correspondence placed dpp-core:Component beneath ceon-product:Product,
which committed every DPPO component to the CEON product-model level and to
the existential composition restrictions that class carries. The accompanying
paper reads dppo:Product as level-neutral, so the axiom was not supported by
the source definitions. It was one of two rows in this registry recorded
without a justification.

Removed from all four artifacts:
- DPPO-CEON.xlsx, the curated mapping row
- DPPO-CEON.ttl, the SSSOM mapping block and the operative subClassOf axiom
- DPPO-CEON-simplified.ttl, the axiom and its owl:Axiom annotation
- DPPO-CEON.rdf, the Alignment API cell

All four now hold ten correspondences and parse cleanly. DPPO-CEON.pdf has not
been regenerated, and the generator notebook has not been re-run.
</commit_message>
<xml_diff>
--- a/mappings/DPPO-CEON/DPPO-CEON.xlsx
+++ b/mappings/DPPO-CEON/DPPO-CEON.xlsx
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" style="1" min="1" max="1"/>
@@ -1031,7 +1031,7 @@
     <row r="8" ht="28.8" customFormat="1" customHeight="1" s="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>DPPO_CEON_0008</t>
+          <t>DPPO_CEON_0010</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -1046,17 +1046,17 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>http://w3id.org/dppo/ontology/dpp-core/Component</t>
+          <t>http://w3id.org/dppo/ontology/dpp-info/DPPInformation</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>dpp-core</t>
+          <t>dpp-info</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>DPPInformation</t>
         </is>
       </c>
       <c r="G8" s="1" t="inlineStr">
@@ -1071,17 +1071,17 @@
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>http://w3id.org/CEON/ontology/product/Product</t>
+          <t>http://w3id.org/CEON/ontology/resourceODP/Information</t>
         </is>
       </c>
       <c r="J8" s="1" t="inlineStr">
         <is>
-          <t>ceon-product</t>
+          <t>resourceODP</t>
         </is>
       </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="L8" s="1" t="inlineStr">
@@ -1096,14 +1096,14 @@
       </c>
       <c r="N8" s="1" t="inlineStr">
         <is>
-          <t>CEON does not define a separate component class; components are products related through ceon-product:hasProductComponent. DPPO's Component, itself a subclass of dpp-odp:Product, is therefore aligned as a specialisation of ceon-product:Product. Stated in the Product Component and Partonomy Alignment section of the accompanying paper.</t>
+          <t>DPPO's DPPInformation is a piece of information contained in a DPP and about a product; CEON's resourceODP:Information is the general notion of information about a resource. Stated in the Digital Product Passport as Document section of the accompanying paper.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>DPPO_CEON_0010</t>
+          <t>DPPO_CEON_0011</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -1113,12 +1113,12 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>Class</t>
+          <t>ObjectProperty</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>http://w3id.org/dppo/ontology/dpp-info/DPPInformation</t>
+          <t>http://w3id.org/dppo/ontology/dpp-info/containsInformation</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>DPPInformation</t>
+          <t>containsInformation</t>
         </is>
       </c>
       <c r="G9" s="1" t="inlineStr">
@@ -1138,12 +1138,12 @@
       </c>
       <c r="H9" s="1" t="inlineStr">
         <is>
-          <t>Class</t>
+          <t>ObjectProperty</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>http://w3id.org/CEON/ontology/resourceODP/Information</t>
+          <t>http://w3id.org/CEON/ontology/resourceODP/containsInformation</t>
         </is>
       </c>
       <c r="J9" s="1" t="inlineStr">
@@ -1153,12 +1153,12 @@
       </c>
       <c r="K9" s="1" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>containsInformation</t>
         </is>
       </c>
       <c r="L9" s="1" t="inlineStr">
         <is>
-          <t>subclass_of</t>
+          <t>subproperty_of</t>
         </is>
       </c>
       <c r="M9" s="1" t="inlineStr">
@@ -1168,14 +1168,14 @@
       </c>
       <c r="N9" s="1" t="inlineStr">
         <is>
-          <t>DPPO's DPPInformation is a piece of information contained in a DPP and about a product; CEON's resourceODP:Information is the general notion of information about a resource. Stated in the Digital Product Passport as Document section of the accompanying paper.</t>
+          <t>DPPO relates a DPP to the pieces of information it contains; the CEON property is the general containment relation between a collection of information and its parts. Stated in the Digital Product Passport as Document section of the accompanying paper.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>DPPO_CEON_0011</t>
+          <t>DPPO_CEON_0012</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -1190,17 +1190,17 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>http://w3id.org/dppo/ontology/dpp-info/containsInformation</t>
+          <t>http://w3id.org/dppo/ontology/dpp-odp/describes</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>dpp-info</t>
+          <t>dpp-odp</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>containsInformation</t>
+          <t>describes</t>
         </is>
       </c>
       <c r="G10" s="1" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>http://w3id.org/CEON/ontology/resourceODP/containsInformation</t>
+          <t>http://w3id.org/CEON/ontology/resourceODP/isAbout</t>
         </is>
       </c>
       <c r="J10" s="1" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="K10" s="1" t="inlineStr">
         <is>
-          <t>containsInformation</t>
+          <t>isAbout</t>
         </is>
       </c>
       <c r="L10" s="1" t="inlineStr">
@@ -1240,14 +1240,14 @@
       </c>
       <c r="N10" s="1" t="inlineStr">
         <is>
-          <t>DPPO relates a DPP to the pieces of information it contains; the CEON property is the general containment relation between a collection of information and its parts. Stated in the Digital Product Passport as Document section of the accompanying paper.</t>
+          <t>Expressed as a subsumption rather than an equivalence to prevent unintended inferences arising from the domain restriction of dpp-odp:describes. Stated in the Digital Product Passport as Document section of the accompanying paper.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>DPPO_CEON_0012</t>
+          <t>DPPO_CEON_0013</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -1262,17 +1262,17 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>http://w3id.org/dppo/ontology/dpp-odp/describes</t>
+          <t>http://w3id.org/dppo/ontology/dpp-info/isAbout</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>dpp-odp</t>
+          <t>dpp-info</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>describes</t>
+          <t>isAbout</t>
         </is>
       </c>
       <c r="G11" s="1" t="inlineStr">
@@ -1312,149 +1312,77 @@
       </c>
       <c r="N11" s="1" t="inlineStr">
         <is>
-          <t>Expressed as a subsumption rather than an equivalence to prevent unintended inferences arising from the domain restriction of dpp-odp:describes. Stated in the Digital Product Passport as Document section of the accompanying paper.</t>
+          <t>Generalises DPPO_CEON_0012: dpp-odp:describes is declared a subproperty of dpp-info:isAbout within DPPO, and both isAbout properties relate a piece of information to the entity it describes. Additional mapping, not discussed in the paper.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>DPPO_CEON_0013</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DPPO_CEON_0015</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>DPPO</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>ObjectProperty</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>http://w3id.org/dppo/ontology/dpp-info/isAbout</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>dpp-info</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>isAbout</t>
-        </is>
-      </c>
-      <c r="G12" s="1" t="inlineStr">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>http://w3id.org/dppo/ontology/dpp-odp/DPP</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>dpp-odp</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>DPP</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>CEON</t>
         </is>
       </c>
-      <c r="H12" s="1" t="inlineStr">
-        <is>
-          <t>ObjectProperty</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>http://w3id.org/CEON/ontology/resourceODP/isAbout</t>
-        </is>
-      </c>
-      <c r="J12" s="1" t="inlineStr">
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>http://w3id.org/CEON/ontology/resourceODP/Information</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>resourceODP</t>
         </is>
       </c>
-      <c r="K12" s="1" t="inlineStr">
-        <is>
-          <t>isAbout</t>
-        </is>
-      </c>
-      <c r="L12" s="1" t="inlineStr">
-        <is>
-          <t>subproperty_of</t>
-        </is>
-      </c>
-      <c r="M12" s="1" t="inlineStr">
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>subclass_of</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
         <is>
           <t>source_to_target</t>
         </is>
       </c>
-      <c r="N12" s="1" t="inlineStr">
-        <is>
-          <t>Generalises DPPO_CEON_0012: dpp-odp:describes is declared a subproperty of dpp-info:isAbout within DPPO, and both isAbout properties relate a piece of information to the entity it describes. Additional mapping, not discussed in the paper.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>DPPO_CEON_0015</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>DPPO</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>http://w3id.org/dppo/ontology/dpp-odp/DPP</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>dpp-odp</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>DPP</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>CEON</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>http://w3id.org/CEON/ontology/resourceODP/Information</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>resourceODP</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Information</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>subclass_of</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>source_to_target</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>CEON defines no passport class. Interpreted within the CEON framework the DPPO passport is a specialised information entity, so it is aligned as a subclass of the CEON information class. An equivalence would be incorrect, because the CEON class covers far more than passports. Stated in the section on the semantic alignment of core classes in the accompanying paper.</t>
         </is>

</xml_diff>